<commit_message>
Nakit akışı şablonu: Kullanım metni sayfa metniyle tutarlı (temizle, E-Tablolar ile açılır)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WoLH5V2Lu6ZNq21Au2PJoE
</commit_message>
<xml_diff>
--- a/foy-nakit-akisi-takip-excel.xlsx
+++ b/foy-nakit-akisi-takip-excel.xlsx
@@ -994,7 +994,7 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dosyada 3 örnek ay var; şablonun çalıştığını görmeniz için kondu. Kendi aylarınızı girmeden önce bu satırları silebilirsiniz.</t>
+          <t xml:space="preserve">Dosyada 3 örnek ay var; şablonun çalıştığını görmeniz için kondu. Kendi aylarınızı girmeden önce bu satırların içeriğini temizleyebilirsiniz (satırı silmeyin, 24 aylık alan daralır).</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1043,7 @@
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">•  Google E-Tablolar'da da açılır ve aynı şekilde hesaplar.</t>
+          <t xml:space="preserve">•  Google E-Tablolar ile de açılır; yalnız temel işlevler kullanılır.</t>
         </is>
       </c>
     </row>

</xml_diff>